<commit_message>
Fix column order to match instruction (A-Z reordered)
Previous order was arbitrary; now matches the .docx spec exactly:
A=*Action, B=*Category, C=*Title, D=Description, E=*ConditionID,
F=PicURL, G=*Quantity, H=*Format, I=*StartPrice, J=*Duration,
K=*Location, L-N=profiles, O=C:Marke, P=C:Produktart,
Q=Custom label (SKU), R=ConditionDescription, S=C:Herstellernummer,
T=C:Produkt, U=C:Modellkompatibilität, V=C:Farbe, W=C:Hersteller,
X=C:Material, Y=C:Markenkompatibilität, Z=C:Installationsart.
Updated COL_MAP, create_template.php, verify_output.php, flat_template.xlsx.

https://claude.ai/code/session_013CC3uQiZgCtv7kaNkq2QqP
</commit_message>
<xml_diff>
--- a/flat_template.xlsx
+++ b/flat_template.xlsx
@@ -20,76 +20,76 @@
     <t>*Action</t>
   </si>
   <si>
+    <t>*Category</t>
+  </si>
+  <si>
+    <t>*Title</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>*ConditionID</t>
+  </si>
+  <si>
+    <t>PicURL</t>
+  </si>
+  <si>
+    <t>*Quantity</t>
+  </si>
+  <si>
+    <t>*Format</t>
+  </si>
+  <si>
+    <t>*StartPrice</t>
+  </si>
+  <si>
+    <t>*Duration</t>
+  </si>
+  <si>
+    <t>*Location</t>
+  </si>
+  <si>
+    <t>ShippingProfileName</t>
+  </si>
+  <si>
+    <t>ReturnProfileName</t>
+  </si>
+  <si>
+    <t>PaymentProfileName</t>
+  </si>
+  <si>
+    <t>C:Marke</t>
+  </si>
+  <si>
+    <t>C:Produktart</t>
+  </si>
+  <si>
     <t>Custom label (SKU)</t>
   </si>
   <si>
-    <t>*Category</t>
-  </si>
-  <si>
-    <t>Description</t>
-  </si>
-  <si>
-    <t>*Title</t>
-  </si>
-  <si>
-    <t>*ConditionID</t>
-  </si>
-  <si>
     <t>ConditionDescription</t>
   </si>
   <si>
-    <t>*StartPrice</t>
-  </si>
-  <si>
-    <t>*Quantity</t>
-  </si>
-  <si>
-    <t>*Format</t>
-  </si>
-  <si>
-    <t>*Duration</t>
-  </si>
-  <si>
-    <t>*Location</t>
-  </si>
-  <si>
-    <t>ShippingProfileName</t>
-  </si>
-  <si>
-    <t>ReturnProfileName</t>
-  </si>
-  <si>
-    <t>PaymentProfileName</t>
-  </si>
-  <si>
-    <t>PicURL</t>
-  </si>
-  <si>
-    <t>C:Marke</t>
+    <t>C:Herstellernummer</t>
+  </si>
+  <si>
+    <t>C:Produkt</t>
+  </si>
+  <si>
+    <t>C:Modellkompatibilität</t>
+  </si>
+  <si>
+    <t>C:Farbe</t>
   </si>
   <si>
     <t>C:Hersteller</t>
   </si>
   <si>
-    <t>C:Produktart</t>
-  </si>
-  <si>
-    <t>C:Produkt</t>
-  </si>
-  <si>
-    <t>C:Farbe</t>
-  </si>
-  <si>
     <t>C:Material</t>
   </si>
   <si>
     <t>C:Markenkompatibilität</t>
-  </si>
-  <si>
-    <t>C:Modellkompatibilität</t>
-  </si>
-  <si>
-    <t>C:Herstellernummer</t>
   </si>
   <si>
     <t>C:Installationsart</t>
@@ -446,30 +446,30 @@
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="9.283" bestFit="true" customWidth="true" style="0"/>
-    <col min="2" max="2" width="22.28" bestFit="true" customWidth="true" style="0"/>
-    <col min="3" max="3" width="11.711" bestFit="true" customWidth="true" style="0"/>
+    <col min="2" max="2" width="11.711" bestFit="true" customWidth="true" style="0"/>
+    <col min="3" max="3" width="8.141" bestFit="true" customWidth="true" style="0"/>
     <col min="4" max="4" width="13.997" bestFit="true" customWidth="true" style="0"/>
-    <col min="5" max="5" width="8.141" bestFit="true" customWidth="true" style="0"/>
-    <col min="6" max="6" width="15.282" bestFit="true" customWidth="true" style="0"/>
-    <col min="7" max="7" width="24.708" bestFit="true" customWidth="true" style="0"/>
-    <col min="8" max="8" width="13.997" bestFit="true" customWidth="true" style="0"/>
-    <col min="9" max="9" width="11.711" bestFit="true" customWidth="true" style="0"/>
-    <col min="10" max="10" width="9.283" bestFit="true" customWidth="true" style="0"/>
+    <col min="5" max="5" width="15.282" bestFit="true" customWidth="true" style="0"/>
+    <col min="6" max="6" width="8.141" bestFit="true" customWidth="true" style="0"/>
+    <col min="7" max="7" width="11.711" bestFit="true" customWidth="true" style="0"/>
+    <col min="8" max="8" width="9.283" bestFit="true" customWidth="true" style="0"/>
+    <col min="9" max="9" width="13.997" bestFit="true" customWidth="true" style="0"/>
+    <col min="10" max="10" width="11.711" bestFit="true" customWidth="true" style="0"/>
     <col min="11" max="11" width="11.711" bestFit="true" customWidth="true" style="0"/>
-    <col min="12" max="12" width="11.711" bestFit="true" customWidth="true" style="0"/>
-    <col min="13" max="13" width="23.423" bestFit="true" customWidth="true" style="0"/>
-    <col min="14" max="14" width="21.138" bestFit="true" customWidth="true" style="0"/>
-    <col min="15" max="15" width="22.28" bestFit="true" customWidth="true" style="0"/>
-    <col min="16" max="16" width="8.141" bestFit="true" customWidth="true" style="0"/>
-    <col min="17" max="17" width="9.283" bestFit="true" customWidth="true" style="0"/>
-    <col min="18" max="18" width="15.282" bestFit="true" customWidth="true" style="0"/>
-    <col min="19" max="19" width="15.282" bestFit="true" customWidth="true" style="0"/>
+    <col min="12" max="12" width="23.423" bestFit="true" customWidth="true" style="0"/>
+    <col min="13" max="13" width="21.138" bestFit="true" customWidth="true" style="0"/>
+    <col min="14" max="14" width="22.28" bestFit="true" customWidth="true" style="0"/>
+    <col min="15" max="15" width="9.283" bestFit="true" customWidth="true" style="0"/>
+    <col min="16" max="16" width="15.282" bestFit="true" customWidth="true" style="0"/>
+    <col min="17" max="17" width="22.28" bestFit="true" customWidth="true" style="0"/>
+    <col min="18" max="18" width="24.708" bestFit="true" customWidth="true" style="0"/>
+    <col min="19" max="19" width="22.28" bestFit="true" customWidth="true" style="0"/>
     <col min="20" max="20" width="11.711" bestFit="true" customWidth="true" style="0"/>
-    <col min="21" max="21" width="9.283" bestFit="true" customWidth="true" style="0"/>
-    <col min="22" max="22" width="12.854" bestFit="true" customWidth="true" style="0"/>
-    <col min="23" max="23" width="26.993" bestFit="true" customWidth="true" style="0"/>
-    <col min="24" max="24" width="26.993" bestFit="true" customWidth="true" style="0"/>
-    <col min="25" max="25" width="22.28" bestFit="true" customWidth="true" style="0"/>
+    <col min="21" max="21" width="26.993" bestFit="true" customWidth="true" style="0"/>
+    <col min="22" max="22" width="9.283" bestFit="true" customWidth="true" style="0"/>
+    <col min="23" max="23" width="15.282" bestFit="true" customWidth="true" style="0"/>
+    <col min="24" max="24" width="12.854" bestFit="true" customWidth="true" style="0"/>
+    <col min="25" max="25" width="26.993" bestFit="true" customWidth="true" style="0"/>
     <col min="26" max="26" width="22.28" bestFit="true" customWidth="true" style="0"/>
   </cols>
   <sheetData>

</xml_diff>